<commit_message>
Change decision variables from DUTIES to ASSIGNMENTS
Change decision variables from DUTIES to ASSIGNMENTS
</commit_message>
<xml_diff>
--- a/test/production/ward_requested_duty_excel.xlsx
+++ b/test/production/ward_requested_duty_excel.xlsx
@@ -16,7 +16,28 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="63">
+  <si>
+    <t>V(1)</t>
+  </si>
+  <si>
+    <t>V(2)</t>
+  </si>
+  <si>
+    <t>V(3)</t>
+  </si>
+  <si>
+    <t>V(4)</t>
+  </si>
+  <si>
+    <t>V(5)</t>
+  </si>
+  <si>
+    <t>V(6)</t>
+  </si>
+  <si>
+    <t>V(7)</t>
+  </si>
   <si>
     <t>C(1)</t>
   </si>
@@ -108,6 +129,15 @@
     <t>LYG(1)</t>
   </si>
   <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>O</t>
+  </si>
+  <si>
     <t>D</t>
   </si>
   <si>
@@ -121,6 +151,9 @@
   </si>
   <si>
     <t>BFY(1)</t>
+  </si>
+  <si>
+    <t>N</t>
   </si>
   <si>
     <t>BFY(2)</t>
@@ -178,10 +211,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11.000000"/>
+      <color theme="9" tint="0"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
@@ -247,20 +286,27 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="20">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf fontId="1" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="1" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf fontId="2" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="3" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="3" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="3" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf fontId="2" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="1" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -760,39 +806,40 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="9.140625"/>
-    <col customWidth="1" min="3" max="7" style="0" width="9.140625"/>
-    <col customWidth="1" min="8" max="8" style="1" width="9.140625"/>
-    <col customWidth="1" min="9" max="14" style="0" width="9.140625"/>
+    <col min="8" max="8" style="1" width="9.140625"/>
+    <col customWidth="1" min="9" max="9" width="9.140625"/>
+    <col customWidth="1" min="10" max="14" style="0" width="9.140625"/>
     <col customWidth="1" min="15" max="15" style="1" width="9.140625"/>
     <col customWidth="1" min="16" max="21" style="0" width="9.140625"/>
     <col customWidth="1" min="22" max="22" style="1" width="9.140625"/>
-    <col customWidth="1" min="23" max="26" style="2" width="9.140625"/>
-    <col min="27" max="28" style="2" width="9.140625"/>
-    <col min="29" max="29" style="1" width="9.140625"/>
-    <col min="30" max="30" style="2" width="9.140625"/>
+    <col customWidth="1" min="23" max="28" style="0" width="9.140625"/>
+    <col customWidth="1" min="29" max="29" style="1" width="9.140625"/>
+    <col customWidth="1" min="30" max="33" style="2" width="9.140625"/>
+    <col min="34" max="35" style="2" width="9.140625"/>
+    <col min="36" max="36" style="1" width="9.140625"/>
+    <col min="37" max="37" style="2" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" s="3" customFormat="1" ht="14.25">
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>6</v>
       </c>
       <c r="I1" s="3" t="s">
@@ -813,7 +860,7 @@
       <c r="N1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="O1" s="6" t="s">
         <v>13</v>
       </c>
       <c r="P1" s="3" t="s">
@@ -834,7 +881,7 @@
       <c r="U1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="V1" s="4" t="s">
+      <c r="V1" s="6" t="s">
         <v>20</v>
       </c>
       <c r="W1" s="3" t="s">
@@ -855,73 +902,129 @@
       <c r="AB1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="AC1" s="4" t="s">
+      <c r="AC1" s="6" t="s">
         <v>27</v>
       </c>
       <c r="AD1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="AE1" s="3"/>
-      <c r="AF1" s="3"/>
-      <c r="AG1" s="3"/>
-      <c r="AH1" s="3"/>
-      <c r="AI1" s="3"/>
-      <c r="AJ1" s="3"/>
+      <c r="AE1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="AF1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="AG1" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="AH1" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="AI1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="AJ1" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="AK1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="AL1" s="3"/>
+      <c r="AM1" s="3"/>
+      <c r="AN1" s="3"/>
+      <c r="AO1" s="3"/>
+      <c r="AP1" s="3"/>
+      <c r="AQ1" s="3"/>
     </row>
     <row r="2" ht="14.25">
       <c r="A2" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="1"/>
-      <c r="I2"/>
-      <c r="J2"/>
-      <c r="K2"/>
+        <v>36</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
-      <c r="N2"/>
+      <c r="N2" s="9"/>
       <c r="O2" s="1"/>
       <c r="P2"/>
       <c r="Q2"/>
-      <c r="R2" s="6" t="s">
-        <v>30</v>
-      </c>
+      <c r="R2"/>
       <c r="S2" s="2"/>
       <c r="T2" s="2"/>
-      <c r="U2" s="6" t="s">
-        <v>30</v>
-      </c>
+      <c r="U2"/>
       <c r="V2" s="1"/>
       <c r="W2"/>
       <c r="X2"/>
-      <c r="Y2"/>
+      <c r="Y2" s="10" t="s">
+        <v>40</v>
+      </c>
       <c r="Z2" s="2"/>
       <c r="AA2" s="2"/>
-      <c r="AB2" s="6" t="s">
-        <v>30</v>
+      <c r="AB2" s="10" t="s">
+        <v>40</v>
       </c>
       <c r="AC2" s="1"/>
-      <c r="AD2" s="2"/>
+      <c r="AD2"/>
+      <c r="AE2"/>
+      <c r="AF2"/>
+      <c r="AG2" s="2"/>
+      <c r="AH2" s="2"/>
+      <c r="AI2" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="AJ2" s="1"/>
+      <c r="AK2" s="2"/>
     </row>
     <row r="3" ht="14.25">
       <c r="A3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3"/>
-      <c r="H3" s="1"/>
-      <c r="I3"/>
-      <c r="J3"/>
-      <c r="K3"/>
+        <v>41</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="J3" s="2"/>
+      <c r="K3" s="10" t="s">
+        <v>40</v>
+      </c>
       <c r="L3" s="2"/>
       <c r="M3" s="2"/>
       <c r="N3"/>
@@ -931,41 +1034,62 @@
       <c r="R3"/>
       <c r="S3" s="2"/>
       <c r="T3" s="2"/>
-      <c r="U3" s="6" t="s">
-        <v>30</v>
-      </c>
+      <c r="U3"/>
       <c r="V3" s="1"/>
       <c r="W3"/>
       <c r="X3"/>
       <c r="Y3"/>
       <c r="Z3" s="2"/>
-      <c r="AA3" s="5"/>
-      <c r="AB3"/>
-      <c r="AC3" s="7"/>
-      <c r="AD3" s="2"/>
+      <c r="AA3" s="2"/>
+      <c r="AB3" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="AC3" s="1"/>
+      <c r="AD3"/>
+      <c r="AE3"/>
+      <c r="AF3"/>
+      <c r="AG3" s="2"/>
+      <c r="AH3" s="9"/>
+      <c r="AI3"/>
+      <c r="AJ3" s="11"/>
+      <c r="AK3" s="2"/>
     </row>
     <row r="4" ht="14.25">
       <c r="A4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4"/>
-      <c r="H4" s="1"/>
-      <c r="I4"/>
-      <c r="J4"/>
-      <c r="K4" s="5"/>
+        <v>42</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="J4" s="2"/>
+      <c r="K4" s="10" t="s">
+        <v>40</v>
+      </c>
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
       <c r="N4"/>
       <c r="O4" s="1"/>
       <c r="P4"/>
       <c r="Q4"/>
-      <c r="R4"/>
+      <c r="R4" s="9"/>
       <c r="S4" s="2"/>
       <c r="T4" s="2"/>
       <c r="U4"/>
@@ -974,77 +1098,119 @@
       <c r="X4"/>
       <c r="Y4"/>
       <c r="Z4" s="2"/>
-      <c r="AA4" s="6" t="s">
-        <v>30</v>
-      </c>
+      <c r="AA4" s="2"/>
       <c r="AB4"/>
       <c r="AC4" s="1"/>
-      <c r="AD4" s="2"/>
+      <c r="AD4"/>
+      <c r="AE4"/>
+      <c r="AF4"/>
+      <c r="AG4" s="2"/>
+      <c r="AH4" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="AI4"/>
+      <c r="AJ4" s="1"/>
+      <c r="AK4" s="2"/>
     </row>
     <row r="5" s="3" customFormat="1" ht="14.25">
       <c r="A5" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="G5" s="3"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="3"/>
+        <v>43</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="H5" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="I5" s="14"/>
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
-      <c r="L5" s="8"/>
-      <c r="M5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="N5" s="3"/>
-      <c r="O5" s="4"/>
+      <c r="O5" s="6"/>
       <c r="P5" s="3"/>
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
-      <c r="S5" s="3"/>
+      <c r="S5" s="14"/>
       <c r="T5" s="3"/>
       <c r="U5" s="3"/>
-      <c r="V5" s="4"/>
+      <c r="V5" s="6"/>
       <c r="W5" s="3"/>
       <c r="X5" s="3"/>
       <c r="Y5" s="3"/>
-      <c r="Z5" s="9" t="s">
-        <v>30</v>
-      </c>
+      <c r="Z5" s="3"/>
       <c r="AA5" s="3"/>
       <c r="AB5" s="3"/>
-      <c r="AC5" s="4"/>
+      <c r="AC5" s="6"/>
       <c r="AD5" s="3"/>
       <c r="AE5" s="3"/>
       <c r="AF5" s="3"/>
-      <c r="AG5" s="3"/>
+      <c r="AG5" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="AH5" s="3"/>
       <c r="AI5" s="3"/>
-      <c r="AJ5" s="3"/>
+      <c r="AJ5" s="6"/>
       <c r="AK5" s="3"/>
       <c r="AL5" s="3"/>
+      <c r="AM5" s="3"/>
+      <c r="AN5" s="3"/>
+      <c r="AO5" s="3"/>
+      <c r="AP5" s="3"/>
+      <c r="AQ5" s="3"/>
+      <c r="AR5" s="3"/>
+      <c r="AS5" s="3"/>
     </row>
     <row r="6" ht="14.25">
       <c r="A6" t="s">
-        <v>34</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="E6" s="5"/>
-      <c r="F6" s="2"/>
-      <c r="G6"/>
-      <c r="H6" s="1"/>
-      <c r="I6"/>
-      <c r="J6"/>
-      <c r="K6"/>
-      <c r="L6" s="2"/>
+        <v>44</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="J6" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="K6" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="L6" s="9"/>
       <c r="M6" s="2"/>
       <c r="N6"/>
       <c r="O6" s="1"/>
@@ -1056,27 +1222,48 @@
       <c r="U6"/>
       <c r="V6" s="1"/>
       <c r="W6"/>
-      <c r="X6" s="5"/>
+      <c r="X6"/>
       <c r="Y6"/>
       <c r="Z6" s="2"/>
       <c r="AA6" s="2"/>
       <c r="AB6"/>
       <c r="AC6" s="1"/>
-      <c r="AD6" s="2"/>
+      <c r="AD6"/>
+      <c r="AE6" s="9"/>
+      <c r="AF6"/>
+      <c r="AG6" s="2"/>
+      <c r="AH6" s="2"/>
+      <c r="AI6"/>
+      <c r="AJ6" s="1"/>
+      <c r="AK6" s="2"/>
     </row>
     <row r="7" ht="14.25">
       <c r="A7" t="s">
-        <v>35</v>
-      </c>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7"/>
-      <c r="H7" s="1"/>
-      <c r="I7"/>
-      <c r="J7"/>
-      <c r="K7"/>
+        <v>46</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
       <c r="N7"/>
@@ -1087,123 +1274,186 @@
       <c r="S7" s="2"/>
       <c r="T7" s="2"/>
       <c r="U7"/>
-      <c r="V7" s="10" t="s">
-        <v>30</v>
-      </c>
+      <c r="V7" s="1"/>
       <c r="W7"/>
       <c r="X7"/>
       <c r="Y7"/>
       <c r="Z7" s="2"/>
       <c r="AA7" s="2"/>
       <c r="AB7"/>
-      <c r="AC7" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="AD7" s="2"/>
+      <c r="AC7" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="AD7"/>
+      <c r="AE7"/>
+      <c r="AF7"/>
+      <c r="AG7" s="2"/>
+      <c r="AH7" s="2"/>
+      <c r="AI7"/>
+      <c r="AJ7" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="AK7" s="2"/>
     </row>
     <row r="8" ht="14.25">
       <c r="A8" t="s">
-        <v>36</v>
-      </c>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8"/>
-      <c r="H8" s="1"/>
-      <c r="I8"/>
-      <c r="J8"/>
-      <c r="K8"/>
-      <c r="L8" s="5"/>
-      <c r="M8" s="5"/>
+        <v>47</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
       <c r="N8"/>
       <c r="O8" s="1"/>
       <c r="P8"/>
-      <c r="Q8" s="6" t="s">
-        <v>30</v>
-      </c>
+      <c r="Q8"/>
       <c r="R8"/>
-      <c r="S8" s="2"/>
-      <c r="T8" s="2"/>
+      <c r="S8" s="9"/>
+      <c r="T8" s="9"/>
       <c r="U8"/>
       <c r="V8" s="1"/>
       <c r="W8"/>
-      <c r="X8"/>
+      <c r="X8" s="10" t="s">
+        <v>40</v>
+      </c>
       <c r="Y8"/>
       <c r="Z8" s="2"/>
       <c r="AA8" s="2"/>
-      <c r="AB8" s="6" t="s">
-        <v>30</v>
-      </c>
+      <c r="AB8"/>
       <c r="AC8" s="1"/>
-      <c r="AD8" s="2"/>
+      <c r="AD8"/>
+      <c r="AE8"/>
+      <c r="AF8"/>
+      <c r="AG8" s="2"/>
+      <c r="AH8" s="2"/>
+      <c r="AI8" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="AJ8" s="1"/>
+      <c r="AK8" s="2"/>
     </row>
     <row r="9" s="3" customFormat="1" ht="14.25">
       <c r="A9" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B9" s="3"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="H9" s="4"/>
+        <v>48</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="H9" s="13" t="s">
+        <v>39</v>
+      </c>
       <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
+      <c r="J9" s="14"/>
+      <c r="K9" s="14"/>
       <c r="L9" s="3"/>
       <c r="M9" s="3"/>
-      <c r="N9" s="3"/>
-      <c r="O9" s="4"/>
+      <c r="N9" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="O9" s="6"/>
       <c r="P9" s="3"/>
       <c r="Q9" s="3"/>
       <c r="R9" s="3"/>
       <c r="S9" s="3"/>
       <c r="T9" s="3"/>
       <c r="U9" s="3"/>
-      <c r="V9" s="4"/>
+      <c r="V9" s="6"/>
       <c r="W9" s="3"/>
       <c r="X9" s="3"/>
       <c r="Y9" s="3"/>
-      <c r="Z9" s="9" t="s">
-        <v>30</v>
-      </c>
+      <c r="Z9" s="3"/>
       <c r="AA9" s="3"/>
       <c r="AB9" s="3"/>
-      <c r="AC9" s="4"/>
+      <c r="AC9" s="6"/>
       <c r="AD9" s="3"/>
       <c r="AE9" s="3"/>
       <c r="AF9" s="3"/>
-      <c r="AG9" s="3"/>
+      <c r="AG9" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="AH9" s="3"/>
       <c r="AI9" s="3"/>
-      <c r="AJ9" s="3"/>
+      <c r="AJ9" s="6"/>
       <c r="AK9" s="3"/>
       <c r="AL9" s="3"/>
       <c r="AM9" s="3"/>
+      <c r="AN9" s="3"/>
+      <c r="AO9" s="3"/>
+      <c r="AP9" s="3"/>
+      <c r="AQ9" s="3"/>
+      <c r="AR9" s="3"/>
+      <c r="AS9" s="3"/>
+      <c r="AT9" s="3"/>
     </row>
     <row r="10" ht="14.25">
       <c r="A10" t="s">
-        <v>38</v>
-      </c>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10"/>
-      <c r="H10" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="I10"/>
-      <c r="J10"/>
-      <c r="K10"/>
+        <v>49</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
       <c r="N10"/>
-      <c r="O10" s="1"/>
+      <c r="O10" s="16" t="s">
+        <v>40</v>
+      </c>
       <c r="P10"/>
       <c r="Q10"/>
       <c r="R10"/>
@@ -1218,27 +1468,46 @@
       <c r="AA10" s="2"/>
       <c r="AB10"/>
       <c r="AC10" s="1"/>
-      <c r="AD10" s="2"/>
+      <c r="AD10"/>
+      <c r="AE10"/>
+      <c r="AF10"/>
+      <c r="AG10" s="2"/>
+      <c r="AH10" s="2"/>
+      <c r="AI10"/>
+      <c r="AJ10" s="1"/>
+      <c r="AK10" s="2"/>
     </row>
     <row r="11" ht="14.25">
       <c r="A11" t="s">
-        <v>39</v>
-      </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="H11" s="1"/>
-      <c r="I11"/>
-      <c r="J11"/>
-      <c r="K11"/>
+        <v>50</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="H11" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
       <c r="L11" s="2"/>
-      <c r="M11" s="2"/>
-      <c r="N11" s="6" t="s">
-        <v>30</v>
+      <c r="M11" s="9"/>
+      <c r="N11" s="10" t="s">
+        <v>40</v>
       </c>
       <c r="O11" s="1"/>
       <c r="P11"/>
@@ -1246,7 +1515,9 @@
       <c r="R11"/>
       <c r="S11" s="2"/>
       <c r="T11" s="2"/>
-      <c r="U11"/>
+      <c r="U11" s="10" t="s">
+        <v>40</v>
+      </c>
       <c r="V11" s="1"/>
       <c r="W11"/>
       <c r="X11"/>
@@ -1255,149 +1526,219 @@
       <c r="AA11" s="2"/>
       <c r="AB11"/>
       <c r="AC11" s="1"/>
-      <c r="AD11" s="2"/>
+      <c r="AD11"/>
+      <c r="AE11"/>
+      <c r="AF11"/>
+      <c r="AG11" s="2"/>
+      <c r="AH11" s="2"/>
+      <c r="AI11"/>
+      <c r="AJ11" s="1"/>
+      <c r="AK11" s="2"/>
     </row>
     <row r="12" ht="14.25">
       <c r="A12" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" s="2"/>
-      <c r="D12" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12"/>
-      <c r="H12" s="1"/>
-      <c r="I12"/>
-      <c r="J12"/>
-      <c r="K12"/>
+        <v>51</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="J12" s="2"/>
+      <c r="K12" s="10" t="s">
+        <v>40</v>
+      </c>
       <c r="L12" s="2"/>
-      <c r="M12" s="5"/>
+      <c r="M12" s="2"/>
       <c r="N12"/>
       <c r="O12" s="1"/>
       <c r="P12"/>
       <c r="Q12"/>
       <c r="R12"/>
-      <c r="S12" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="T12" s="2"/>
+      <c r="S12" s="2"/>
+      <c r="T12" s="9"/>
       <c r="U12"/>
-      <c r="V12" s="7"/>
+      <c r="V12" s="1"/>
       <c r="W12"/>
       <c r="X12"/>
       <c r="Y12"/>
-      <c r="Z12" s="2"/>
+      <c r="Z12" s="10" t="s">
+        <v>40</v>
+      </c>
       <c r="AA12" s="2"/>
       <c r="AB12"/>
-      <c r="AC12" s="1"/>
-      <c r="AD12" s="2"/>
+      <c r="AC12" s="11"/>
+      <c r="AD12"/>
+      <c r="AE12"/>
+      <c r="AF12"/>
+      <c r="AG12" s="2"/>
+      <c r="AH12" s="2"/>
+      <c r="AI12"/>
+      <c r="AJ12" s="1"/>
+      <c r="AK12" s="2"/>
     </row>
     <row r="13" ht="14.25">
       <c r="A13" t="s">
-        <v>41</v>
-      </c>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="F13" s="2"/>
-      <c r="G13"/>
-      <c r="H13" s="1"/>
-      <c r="I13"/>
-      <c r="J13"/>
-      <c r="K13"/>
-      <c r="L13" s="2"/>
+        <v>52</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="H13" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
+      <c r="L13" s="10" t="s">
+        <v>40</v>
+      </c>
       <c r="M13" s="2"/>
       <c r="N13"/>
-      <c r="O13" s="7"/>
+      <c r="O13" s="1"/>
       <c r="P13"/>
       <c r="Q13"/>
       <c r="R13"/>
       <c r="S13" s="2"/>
       <c r="T13" s="2"/>
       <c r="U13"/>
-      <c r="V13" s="1"/>
+      <c r="V13" s="11"/>
       <c r="W13"/>
       <c r="X13"/>
-      <c r="Y13" s="6" t="s">
-        <v>30</v>
-      </c>
+      <c r="Y13"/>
       <c r="Z13" s="2"/>
       <c r="AA13" s="2"/>
       <c r="AB13"/>
       <c r="AC13" s="1"/>
-      <c r="AD13" s="2"/>
+      <c r="AD13"/>
+      <c r="AE13"/>
+      <c r="AF13" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="AG13" s="2"/>
+      <c r="AH13" s="2"/>
+      <c r="AI13"/>
+      <c r="AJ13" s="1"/>
+      <c r="AK13" s="2"/>
     </row>
     <row r="14" s="3" customFormat="1" ht="14.25">
       <c r="A14" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="4"/>
+        <v>53</v>
+      </c>
+      <c r="B14" s="12"/>
+      <c r="C14" s="12"/>
+      <c r="D14" s="12"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="12"/>
+      <c r="G14" s="12"/>
+      <c r="H14" s="13"/>
       <c r="I14" s="3"/>
-      <c r="J14" s="8"/>
+      <c r="J14" s="3"/>
       <c r="K14" s="3"/>
       <c r="L14" s="3"/>
       <c r="M14" s="3"/>
       <c r="N14" s="3"/>
-      <c r="O14" s="11" t="s">
-        <v>30</v>
-      </c>
+      <c r="O14" s="6"/>
       <c r="P14" s="3"/>
-      <c r="Q14" s="3"/>
+      <c r="Q14" s="14"/>
       <c r="R14" s="3"/>
       <c r="S14" s="3"/>
       <c r="T14" s="3"/>
       <c r="U14" s="3"/>
-      <c r="V14" s="12"/>
+      <c r="V14" s="17" t="s">
+        <v>40</v>
+      </c>
       <c r="W14" s="3"/>
       <c r="X14" s="3"/>
       <c r="Y14" s="3"/>
       <c r="Z14" s="3"/>
       <c r="AA14" s="3"/>
-      <c r="AB14" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="AC14" s="4"/>
+      <c r="AB14" s="3"/>
+      <c r="AC14" s="18"/>
       <c r="AD14" s="3"/>
       <c r="AE14" s="3"/>
       <c r="AF14" s="3"/>
       <c r="AG14" s="3"/>
       <c r="AH14" s="3"/>
-      <c r="AI14" s="3"/>
-      <c r="AJ14" s="3"/>
+      <c r="AI14" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="AJ14" s="6"/>
       <c r="AK14" s="3"/>
       <c r="AL14" s="3"/>
+      <c r="AM14" s="3"/>
+      <c r="AN14" s="3"/>
+      <c r="AO14" s="3"/>
+      <c r="AP14" s="3"/>
+      <c r="AQ14" s="3"/>
+      <c r="AR14" s="3"/>
+      <c r="AS14" s="3"/>
     </row>
     <row r="15" ht="14.25">
       <c r="A15" t="s">
-        <v>43</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="H15" s="1"/>
-      <c r="I15"/>
-      <c r="J15"/>
-      <c r="K15"/>
+        <v>54</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="I15" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
       <c r="L15" s="2"/>
       <c r="M15" s="2"/>
-      <c r="N15"/>
+      <c r="N15" s="10" t="s">
+        <v>40</v>
+      </c>
       <c r="O15" s="1"/>
       <c r="P15"/>
       <c r="Q15"/>
@@ -1413,26 +1754,47 @@
       <c r="AA15" s="2"/>
       <c r="AB15"/>
       <c r="AC15" s="1"/>
-      <c r="AD15" s="2"/>
+      <c r="AD15"/>
+      <c r="AE15"/>
+      <c r="AF15"/>
+      <c r="AG15" s="2"/>
+      <c r="AH15" s="2"/>
+      <c r="AI15"/>
+      <c r="AJ15" s="1"/>
+      <c r="AK15" s="2"/>
     </row>
     <row r="16" ht="14.25">
       <c r="A16" t="s">
-        <v>44</v>
-      </c>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="5"/>
-      <c r="J16"/>
-      <c r="K16"/>
+        <v>55</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="H16" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
       <c r="N16"/>
       <c r="O16" s="1"/>
-      <c r="P16"/>
+      <c r="P16" s="9"/>
       <c r="Q16"/>
       <c r="R16"/>
       <c r="S16" s="2"/>
@@ -1446,73 +1808,115 @@
       <c r="AA16" s="2"/>
       <c r="AB16"/>
       <c r="AC16" s="1"/>
-      <c r="AD16" s="2"/>
+      <c r="AD16"/>
+      <c r="AE16"/>
+      <c r="AF16"/>
+      <c r="AG16" s="2"/>
+      <c r="AH16" s="2"/>
+      <c r="AI16"/>
+      <c r="AJ16" s="1"/>
+      <c r="AK16" s="2"/>
     </row>
     <row r="17" ht="14.25">
       <c r="A17" t="s">
+        <v>56</v>
+      </c>
+      <c r="B17" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="H17" s="1"/>
-      <c r="I17"/>
-      <c r="J17"/>
-      <c r="K17"/>
+      <c r="C17" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="H17" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="J17" s="2"/>
+      <c r="K17" s="2"/>
       <c r="L17" s="2"/>
       <c r="M17" s="2"/>
-      <c r="N17"/>
-      <c r="O17" s="7"/>
+      <c r="N17" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="O17" s="1"/>
       <c r="P17"/>
       <c r="Q17"/>
       <c r="R17"/>
       <c r="S17" s="2"/>
       <c r="T17" s="2"/>
       <c r="U17"/>
-      <c r="V17" s="1"/>
-      <c r="W17" s="6" t="s">
-        <v>30</v>
-      </c>
+      <c r="V17" s="11"/>
+      <c r="W17"/>
       <c r="X17"/>
       <c r="Y17"/>
       <c r="Z17" s="2"/>
       <c r="AA17" s="2"/>
       <c r="AB17"/>
-      <c r="AC17" s="7"/>
-      <c r="AD17" s="2"/>
+      <c r="AC17" s="1"/>
+      <c r="AD17" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="AE17"/>
+      <c r="AF17"/>
+      <c r="AG17" s="2"/>
+      <c r="AH17" s="2"/>
+      <c r="AI17"/>
+      <c r="AJ17" s="11"/>
+      <c r="AK17" s="2"/>
     </row>
     <row r="18" ht="14.25">
       <c r="A18" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="I18" s="5"/>
-      <c r="J18"/>
-      <c r="K18"/>
+        <v>57</v>
+      </c>
+      <c r="B18" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C18" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="D18" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="E18" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="F18" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="G18" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="H18" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
       <c r="L18" s="2"/>
       <c r="M18" s="2"/>
-      <c r="N18" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="O18" s="1"/>
-      <c r="P18"/>
+      <c r="N18" s="10"/>
+      <c r="O18" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="P18" s="9"/>
       <c r="Q18"/>
       <c r="R18"/>
       <c r="S18" s="2"/>
       <c r="T18" s="2"/>
-      <c r="U18"/>
+      <c r="U18" s="10" t="s">
+        <v>40</v>
+      </c>
       <c r="V18" s="1"/>
       <c r="W18"/>
       <c r="X18"/>
@@ -1521,67 +1925,95 @@
       <c r="AA18" s="2"/>
       <c r="AB18"/>
       <c r="AC18" s="1"/>
-      <c r="AD18" s="2"/>
+      <c r="AD18"/>
+      <c r="AE18"/>
+      <c r="AF18"/>
+      <c r="AG18" s="2"/>
+      <c r="AH18" s="2"/>
+      <c r="AI18"/>
+      <c r="AJ18" s="1"/>
+      <c r="AK18" s="2"/>
     </row>
     <row r="19" s="3" customFormat="1" ht="14.25">
       <c r="A19" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="4"/>
+        <v>58</v>
+      </c>
+      <c r="B19" s="12"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="13"/>
       <c r="I19" s="3"/>
       <c r="J19" s="3"/>
       <c r="K19" s="3"/>
       <c r="L19" s="3"/>
       <c r="M19" s="3"/>
       <c r="N19" s="3"/>
-      <c r="O19" s="12"/>
+      <c r="O19" s="6"/>
       <c r="P19" s="3"/>
       <c r="Q19" s="3"/>
       <c r="R19" s="3"/>
-      <c r="S19" s="9" t="s">
-        <v>30</v>
-      </c>
+      <c r="S19" s="3"/>
       <c r="T19" s="3"/>
       <c r="U19" s="3"/>
-      <c r="V19" s="12"/>
+      <c r="V19" s="18"/>
       <c r="W19" s="3"/>
       <c r="X19" s="3"/>
       <c r="Y19" s="3"/>
-      <c r="Z19" s="3"/>
+      <c r="Z19" s="15" t="s">
+        <v>40</v>
+      </c>
       <c r="AA19" s="3"/>
       <c r="AB19" s="3"/>
-      <c r="AC19" s="4"/>
+      <c r="AC19" s="18"/>
       <c r="AD19" s="3"/>
       <c r="AE19" s="3"/>
       <c r="AF19" s="3"/>
       <c r="AG19" s="3"/>
       <c r="AH19" s="3"/>
       <c r="AI19" s="3"/>
-      <c r="AJ19" s="3"/>
+      <c r="AJ19" s="6"/>
       <c r="AK19" s="3"/>
       <c r="AL19" s="3"/>
+      <c r="AM19" s="3"/>
+      <c r="AN19" s="3"/>
+      <c r="AO19" s="3"/>
+      <c r="AP19" s="3"/>
+      <c r="AQ19" s="3"/>
+      <c r="AR19" s="3"/>
+      <c r="AS19" s="3"/>
     </row>
     <row r="20" ht="14.25">
       <c r="A20" t="s">
-        <v>48</v>
-      </c>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="5"/>
-      <c r="G20"/>
-      <c r="H20" s="1"/>
-      <c r="I20"/>
-      <c r="J20"/>
-      <c r="K20"/>
+        <v>59</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H20" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="J20" s="2"/>
+      <c r="K20" s="2"/>
       <c r="L20" s="2"/>
-      <c r="M20" s="2"/>
+      <c r="M20" s="9"/>
       <c r="N20"/>
       <c r="O20" s="1"/>
       <c r="P20"/>
@@ -1595,24 +2027,45 @@
       <c r="X20"/>
       <c r="Y20"/>
       <c r="Z20" s="2"/>
-      <c r="AA20" s="5"/>
+      <c r="AA20" s="2"/>
       <c r="AB20"/>
       <c r="AC20" s="1"/>
-      <c r="AD20" s="2"/>
+      <c r="AD20"/>
+      <c r="AE20"/>
+      <c r="AF20"/>
+      <c r="AG20" s="2"/>
+      <c r="AH20" s="9"/>
+      <c r="AI20"/>
+      <c r="AJ20" s="1"/>
+      <c r="AK20" s="2"/>
     </row>
     <row r="21" ht="14.25">
       <c r="A21" t="s">
-        <v>49</v>
-      </c>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21"/>
-      <c r="H21" s="1"/>
-      <c r="I21"/>
-      <c r="J21"/>
-      <c r="K21"/>
+        <v>60</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="H21" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
       <c r="N21"/>
@@ -1626,60 +2079,102 @@
       <c r="V21" s="1"/>
       <c r="W21"/>
       <c r="X21"/>
-      <c r="Y21" s="5"/>
+      <c r="Y21"/>
       <c r="Z21" s="2"/>
       <c r="AA21" s="2"/>
       <c r="AB21"/>
-      <c r="AC21" s="7"/>
-      <c r="AD21" s="2"/>
+      <c r="AC21" s="1"/>
+      <c r="AD21"/>
+      <c r="AE21"/>
+      <c r="AF21" s="9"/>
+      <c r="AG21" s="2"/>
+      <c r="AH21" s="2"/>
+      <c r="AI21"/>
+      <c r="AJ21" s="11"/>
+      <c r="AK21" s="2"/>
     </row>
     <row r="22" ht="14.25">
       <c r="A22" t="s">
-        <v>50</v>
-      </c>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22"/>
-      <c r="H22" s="1"/>
-      <c r="I22"/>
-      <c r="J22"/>
-      <c r="K22"/>
+        <v>61</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="H22" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="J22" s="2"/>
+      <c r="K22" s="2"/>
       <c r="L22" s="2"/>
-      <c r="M22" s="5"/>
+      <c r="M22" s="2"/>
       <c r="N22"/>
       <c r="O22" s="1"/>
-      <c r="P22" s="5"/>
+      <c r="P22"/>
       <c r="Q22"/>
       <c r="R22"/>
       <c r="S22" s="2"/>
-      <c r="T22" s="2"/>
+      <c r="T22" s="9"/>
       <c r="U22"/>
       <c r="V22" s="1"/>
-      <c r="W22"/>
+      <c r="W22" s="9"/>
       <c r="X22"/>
       <c r="Y22"/>
       <c r="Z22" s="2"/>
       <c r="AA22" s="2"/>
       <c r="AB22"/>
       <c r="AC22" s="1"/>
-      <c r="AD22" s="2"/>
+      <c r="AD22"/>
+      <c r="AE22"/>
+      <c r="AF22"/>
+      <c r="AG22" s="2"/>
+      <c r="AH22" s="2"/>
+      <c r="AI22"/>
+      <c r="AJ22" s="1"/>
+      <c r="AK22" s="2"/>
     </row>
     <row r="23" ht="14.25">
       <c r="A23" t="s">
-        <v>51</v>
-      </c>
-      <c r="B23" s="5"/>
-      <c r="C23" s="5"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23"/>
-      <c r="H23" s="1"/>
-      <c r="I23"/>
-      <c r="J23"/>
-      <c r="K23"/>
+        <v>62</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="H23" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="I23" s="9"/>
+      <c r="J23" s="9"/>
+      <c r="K23" s="2"/>
       <c r="L23" s="2"/>
       <c r="M23" s="2"/>
       <c r="N23"/>
@@ -1698,16 +2193,16 @@
       <c r="AA23" s="2"/>
       <c r="AB23"/>
       <c r="AC23" s="1"/>
-      <c r="AD23" s="2"/>
+      <c r="AD23"/>
+      <c r="AE23"/>
+      <c r="AF23"/>
+      <c r="AG23" s="2"/>
+      <c r="AH23" s="2"/>
+      <c r="AI23"/>
+      <c r="AJ23" s="1"/>
+      <c r="AK23" s="2"/>
     </row>
     <row r="24" ht="14.25">
-      <c r="C24"/>
-      <c r="D24"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24"/>
-      <c r="H24" s="1"/>
-      <c r="I24"/>
       <c r="J24"/>
       <c r="K24"/>
       <c r="L24" s="2"/>
@@ -1728,16 +2223,16 @@
       <c r="AA24" s="2"/>
       <c r="AB24"/>
       <c r="AC24" s="1"/>
-      <c r="AD24" s="2"/>
+      <c r="AD24"/>
+      <c r="AE24"/>
+      <c r="AF24"/>
+      <c r="AG24" s="2"/>
+      <c r="AH24" s="2"/>
+      <c r="AI24"/>
+      <c r="AJ24" s="1"/>
+      <c r="AK24" s="2"/>
     </row>
     <row r="25" ht="14.25">
-      <c r="C25"/>
-      <c r="D25"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25"/>
-      <c r="H25" s="1"/>
-      <c r="I25"/>
       <c r="J25"/>
       <c r="K25"/>
       <c r="L25" s="2"/>
@@ -1758,16 +2253,16 @@
       <c r="AA25" s="2"/>
       <c r="AB25"/>
       <c r="AC25" s="1"/>
-      <c r="AD25" s="2"/>
+      <c r="AD25"/>
+      <c r="AE25"/>
+      <c r="AF25"/>
+      <c r="AG25" s="2"/>
+      <c r="AH25" s="2"/>
+      <c r="AI25"/>
+      <c r="AJ25" s="1"/>
+      <c r="AK25" s="2"/>
     </row>
     <row r="26" ht="14.25">
-      <c r="C26"/>
-      <c r="D26"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26"/>
-      <c r="H26" s="1"/>
-      <c r="I26"/>
       <c r="J26"/>
       <c r="K26"/>
       <c r="L26" s="2"/>
@@ -1788,16 +2283,16 @@
       <c r="AA26" s="2"/>
       <c r="AB26"/>
       <c r="AC26" s="1"/>
-      <c r="AD26" s="2"/>
+      <c r="AD26"/>
+      <c r="AE26"/>
+      <c r="AF26"/>
+      <c r="AG26" s="2"/>
+      <c r="AH26" s="2"/>
+      <c r="AI26"/>
+      <c r="AJ26" s="1"/>
+      <c r="AK26" s="2"/>
     </row>
     <row r="27" ht="14.25">
-      <c r="C27"/>
-      <c r="D27"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27"/>
-      <c r="H27" s="1"/>
-      <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
       <c r="L27" s="2"/>
@@ -1818,16 +2313,16 @@
       <c r="AA27" s="2"/>
       <c r="AB27"/>
       <c r="AC27" s="1"/>
-      <c r="AD27" s="2"/>
+      <c r="AD27"/>
+      <c r="AE27"/>
+      <c r="AF27"/>
+      <c r="AG27" s="2"/>
+      <c r="AH27" s="2"/>
+      <c r="AI27"/>
+      <c r="AJ27" s="1"/>
+      <c r="AK27" s="2"/>
     </row>
     <row r="28" ht="14.25">
-      <c r="C28"/>
-      <c r="D28"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28"/>
-      <c r="H28" s="1"/>
-      <c r="I28"/>
       <c r="J28"/>
       <c r="K28"/>
       <c r="L28" s="2"/>
@@ -1848,16 +2343,16 @@
       <c r="AA28" s="2"/>
       <c r="AB28"/>
       <c r="AC28" s="1"/>
-      <c r="AD28" s="2"/>
+      <c r="AD28"/>
+      <c r="AE28"/>
+      <c r="AF28"/>
+      <c r="AG28" s="2"/>
+      <c r="AH28" s="2"/>
+      <c r="AI28"/>
+      <c r="AJ28" s="1"/>
+      <c r="AK28" s="2"/>
     </row>
     <row r="29" ht="14.25">
-      <c r="C29"/>
-      <c r="D29"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29"/>
-      <c r="H29" s="1"/>
-      <c r="I29"/>
       <c r="J29"/>
       <c r="K29"/>
       <c r="L29" s="2"/>
@@ -1878,16 +2373,16 @@
       <c r="AA29" s="2"/>
       <c r="AB29"/>
       <c r="AC29" s="1"/>
-      <c r="AD29" s="2"/>
+      <c r="AD29"/>
+      <c r="AE29"/>
+      <c r="AF29"/>
+      <c r="AG29" s="2"/>
+      <c r="AH29" s="2"/>
+      <c r="AI29"/>
+      <c r="AJ29" s="1"/>
+      <c r="AK29" s="2"/>
     </row>
     <row r="30" ht="14.25">
-      <c r="C30"/>
-      <c r="D30"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30"/>
-      <c r="H30" s="1"/>
-      <c r="I30"/>
       <c r="J30"/>
       <c r="K30"/>
       <c r="L30" s="2"/>
@@ -1908,16 +2403,16 @@
       <c r="AA30" s="2"/>
       <c r="AB30"/>
       <c r="AC30" s="1"/>
-      <c r="AD30" s="2"/>
+      <c r="AD30"/>
+      <c r="AE30"/>
+      <c r="AF30"/>
+      <c r="AG30" s="2"/>
+      <c r="AH30" s="2"/>
+      <c r="AI30"/>
+      <c r="AJ30" s="1"/>
+      <c r="AK30" s="2"/>
     </row>
     <row r="31" ht="14.25">
-      <c r="C31"/>
-      <c r="D31"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-      <c r="G31"/>
-      <c r="H31" s="1"/>
-      <c r="I31"/>
       <c r="J31"/>
       <c r="K31"/>
       <c r="L31" s="2"/>
@@ -1938,16 +2433,16 @@
       <c r="AA31" s="2"/>
       <c r="AB31"/>
       <c r="AC31" s="1"/>
-      <c r="AD31" s="2"/>
+      <c r="AD31"/>
+      <c r="AE31"/>
+      <c r="AF31"/>
+      <c r="AG31" s="2"/>
+      <c r="AH31" s="2"/>
+      <c r="AI31"/>
+      <c r="AJ31" s="1"/>
+      <c r="AK31" s="2"/>
     </row>
     <row r="32" ht="14.25">
-      <c r="C32"/>
-      <c r="D32"/>
-      <c r="E32" s="2"/>
-      <c r="F32" s="2"/>
-      <c r="G32"/>
-      <c r="H32" s="1"/>
-      <c r="I32"/>
       <c r="J32"/>
       <c r="K32"/>
       <c r="L32" s="2"/>
@@ -1968,16 +2463,16 @@
       <c r="AA32" s="2"/>
       <c r="AB32"/>
       <c r="AC32" s="1"/>
-      <c r="AD32" s="2"/>
+      <c r="AD32"/>
+      <c r="AE32"/>
+      <c r="AF32"/>
+      <c r="AG32" s="2"/>
+      <c r="AH32" s="2"/>
+      <c r="AI32"/>
+      <c r="AJ32" s="1"/>
+      <c r="AK32" s="2"/>
     </row>
     <row r="33" ht="14.25">
-      <c r="C33"/>
-      <c r="D33"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33"/>
-      <c r="H33" s="1"/>
-      <c r="I33"/>
       <c r="J33"/>
       <c r="K33"/>
       <c r="L33" s="2"/>
@@ -1998,16 +2493,16 @@
       <c r="AA33" s="2"/>
       <c r="AB33"/>
       <c r="AC33" s="1"/>
-      <c r="AD33" s="2"/>
+      <c r="AD33"/>
+      <c r="AE33"/>
+      <c r="AF33"/>
+      <c r="AG33" s="2"/>
+      <c r="AH33" s="2"/>
+      <c r="AI33"/>
+      <c r="AJ33" s="1"/>
+      <c r="AK33" s="2"/>
     </row>
     <row r="34" ht="14.25">
-      <c r="C34"/>
-      <c r="D34"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-      <c r="G34"/>
-      <c r="H34" s="1"/>
-      <c r="I34"/>
       <c r="J34"/>
       <c r="K34"/>
       <c r="L34" s="2"/>
@@ -2028,16 +2523,16 @@
       <c r="AA34" s="2"/>
       <c r="AB34"/>
       <c r="AC34" s="1"/>
-      <c r="AD34" s="2"/>
+      <c r="AD34"/>
+      <c r="AE34"/>
+      <c r="AF34"/>
+      <c r="AG34" s="2"/>
+      <c r="AH34" s="2"/>
+      <c r="AI34"/>
+      <c r="AJ34" s="1"/>
+      <c r="AK34" s="2"/>
     </row>
     <row r="35" ht="14.25">
-      <c r="C35"/>
-      <c r="D35"/>
-      <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-      <c r="G35"/>
-      <c r="H35" s="1"/>
-      <c r="I35"/>
       <c r="J35"/>
       <c r="K35"/>
       <c r="L35" s="2"/>
@@ -2058,16 +2553,16 @@
       <c r="AA35" s="2"/>
       <c r="AB35"/>
       <c r="AC35" s="1"/>
-      <c r="AD35" s="2"/>
+      <c r="AD35"/>
+      <c r="AE35"/>
+      <c r="AF35"/>
+      <c r="AG35" s="2"/>
+      <c r="AH35" s="2"/>
+      <c r="AI35"/>
+      <c r="AJ35" s="1"/>
+      <c r="AK35" s="2"/>
     </row>
     <row r="36" ht="14.25">
-      <c r="C36"/>
-      <c r="D36"/>
-      <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-      <c r="G36"/>
-      <c r="H36" s="1"/>
-      <c r="I36"/>
       <c r="J36"/>
       <c r="K36"/>
       <c r="L36" s="2"/>
@@ -2088,16 +2583,16 @@
       <c r="AA36" s="2"/>
       <c r="AB36"/>
       <c r="AC36" s="1"/>
-      <c r="AD36" s="2"/>
+      <c r="AD36"/>
+      <c r="AE36"/>
+      <c r="AF36"/>
+      <c r="AG36" s="2"/>
+      <c r="AH36" s="2"/>
+      <c r="AI36"/>
+      <c r="AJ36" s="1"/>
+      <c r="AK36" s="2"/>
     </row>
     <row r="37" ht="14.25">
-      <c r="C37"/>
-      <c r="D37"/>
-      <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
-      <c r="G37"/>
-      <c r="H37" s="1"/>
-      <c r="I37"/>
       <c r="J37"/>
       <c r="K37"/>
       <c r="L37" s="2"/>
@@ -2118,16 +2613,16 @@
       <c r="AA37" s="2"/>
       <c r="AB37"/>
       <c r="AC37" s="1"/>
-      <c r="AD37" s="2"/>
+      <c r="AD37"/>
+      <c r="AE37"/>
+      <c r="AF37"/>
+      <c r="AG37" s="2"/>
+      <c r="AH37" s="2"/>
+      <c r="AI37"/>
+      <c r="AJ37" s="1"/>
+      <c r="AK37" s="2"/>
     </row>
     <row r="38" ht="14.25">
-      <c r="C38"/>
-      <c r="D38"/>
-      <c r="E38" s="2"/>
-      <c r="F38" s="2"/>
-      <c r="G38"/>
-      <c r="H38" s="1"/>
-      <c r="I38"/>
       <c r="J38"/>
       <c r="K38"/>
       <c r="L38" s="2"/>
@@ -2148,16 +2643,16 @@
       <c r="AA38" s="2"/>
       <c r="AB38"/>
       <c r="AC38" s="1"/>
-      <c r="AD38" s="2"/>
+      <c r="AD38"/>
+      <c r="AE38"/>
+      <c r="AF38"/>
+      <c r="AG38" s="2"/>
+      <c r="AH38" s="2"/>
+      <c r="AI38"/>
+      <c r="AJ38" s="1"/>
+      <c r="AK38" s="2"/>
     </row>
     <row r="39" ht="14.25">
-      <c r="C39"/>
-      <c r="D39"/>
-      <c r="E39" s="2"/>
-      <c r="F39" s="2"/>
-      <c r="G39"/>
-      <c r="H39" s="1"/>
-      <c r="I39"/>
       <c r="J39"/>
       <c r="K39"/>
       <c r="L39" s="2"/>
@@ -2178,16 +2673,16 @@
       <c r="AA39" s="2"/>
       <c r="AB39"/>
       <c r="AC39" s="1"/>
-      <c r="AD39" s="2"/>
+      <c r="AD39"/>
+      <c r="AE39"/>
+      <c r="AF39"/>
+      <c r="AG39" s="2"/>
+      <c r="AH39" s="2"/>
+      <c r="AI39"/>
+      <c r="AJ39" s="1"/>
+      <c r="AK39" s="2"/>
     </row>
     <row r="40" ht="14.25">
-      <c r="C40"/>
-      <c r="D40"/>
-      <c r="E40" s="2"/>
-      <c r="F40" s="2"/>
-      <c r="G40"/>
-      <c r="H40" s="1"/>
-      <c r="I40"/>
       <c r="J40"/>
       <c r="K40"/>
       <c r="L40" s="2"/>
@@ -2208,16 +2703,16 @@
       <c r="AA40" s="2"/>
       <c r="AB40"/>
       <c r="AC40" s="1"/>
-      <c r="AD40" s="2"/>
+      <c r="AD40"/>
+      <c r="AE40"/>
+      <c r="AF40"/>
+      <c r="AG40" s="2"/>
+      <c r="AH40" s="2"/>
+      <c r="AI40"/>
+      <c r="AJ40" s="1"/>
+      <c r="AK40" s="2"/>
     </row>
     <row r="41" ht="14.25">
-      <c r="C41"/>
-      <c r="D41"/>
-      <c r="E41" s="2"/>
-      <c r="F41" s="2"/>
-      <c r="G41"/>
-      <c r="H41" s="1"/>
-      <c r="I41"/>
       <c r="J41"/>
       <c r="K41"/>
       <c r="L41" s="2"/>
@@ -2238,16 +2733,16 @@
       <c r="AA41" s="2"/>
       <c r="AB41"/>
       <c r="AC41" s="1"/>
-      <c r="AD41" s="2"/>
+      <c r="AD41"/>
+      <c r="AE41"/>
+      <c r="AF41"/>
+      <c r="AG41" s="2"/>
+      <c r="AH41" s="2"/>
+      <c r="AI41"/>
+      <c r="AJ41" s="1"/>
+      <c r="AK41" s="2"/>
     </row>
     <row r="42" ht="14.25">
-      <c r="C42"/>
-      <c r="D42"/>
-      <c r="E42" s="2"/>
-      <c r="F42" s="2"/>
-      <c r="G42"/>
-      <c r="H42" s="1"/>
-      <c r="I42"/>
       <c r="J42"/>
       <c r="K42"/>
       <c r="L42" s="2"/>
@@ -2268,7 +2763,14 @@
       <c r="AA42" s="2"/>
       <c r="AB42"/>
       <c r="AC42" s="1"/>
-      <c r="AD42" s="2"/>
+      <c r="AD42"/>
+      <c r="AE42"/>
+      <c r="AF42"/>
+      <c r="AG42" s="2"/>
+      <c r="AH42" s="2"/>
+      <c r="AI42"/>
+      <c r="AJ42" s="1"/>
+      <c r="AK42" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>

</xml_diff>

<commit_message>
Show roster at class level to debug MAX_WARD
Show roster at class level to debug MAX_WARD
</commit_message>
<xml_diff>
--- a/test/production/ward_requested_duty_excel.xlsx
+++ b/test/production/ward_requested_duty_excel.xlsx
@@ -214,7 +214,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -239,6 +239,12 @@
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11.000000"/>
+      <color indexed="2"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -248,7 +254,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -285,17 +291,27 @@
       </bottom>
       <diagonal style="none"/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
@@ -306,6 +322,11 @@
     <xf fontId="2" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf fontId="3" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf fontId="3" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="4" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="4" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="4" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="4" fillId="0" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf fontId="3" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf fontId="2" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
@@ -930,7 +951,7 @@
       <c r="AK1" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="AL1" s="5" t="s">
+      <c r="AL1" s="3" t="s">
         <v>36</v>
       </c>
       <c r="AM1" s="3"/>
@@ -943,32 +964,32 @@
       <c r="A2" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C2" s="6" t="s">
+      <c r="B2" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D2" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="F2" s="6" t="s">
+      <c r="D2" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="6" t="s">
         <v>40</v>
       </c>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
-      <c r="N2" s="8"/>
+      <c r="N2" s="7"/>
       <c r="O2" s="1"/>
       <c r="P2"/>
       <c r="Q2"/>
@@ -979,12 +1000,12 @@
       <c r="V2" s="1"/>
       <c r="W2"/>
       <c r="X2"/>
-      <c r="Y2" s="9" t="s">
+      <c r="Y2" s="8" t="s">
         <v>41</v>
       </c>
       <c r="Z2" s="2"/>
       <c r="AA2" s="2"/>
-      <c r="AB2" s="9" t="s">
+      <c r="AB2" s="8" t="s">
         <v>41</v>
       </c>
       <c r="AC2" s="1"/>
@@ -993,7 +1014,7 @@
       <c r="AF2"/>
       <c r="AG2" s="2"/>
       <c r="AH2" s="2"/>
-      <c r="AI2" s="9" t="s">
+      <c r="AI2" s="8" t="s">
         <v>41</v>
       </c>
       <c r="AJ2" s="1"/>
@@ -1003,29 +1024,29 @@
       <c r="A3" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="H3" s="7" t="s">
+      <c r="B3" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="H3" s="6" t="s">
         <v>40</v>
       </c>
       <c r="J3" s="2"/>
-      <c r="K3" s="9" t="s">
+      <c r="K3" s="8" t="s">
         <v>41</v>
       </c>
       <c r="L3" s="2"/>
@@ -1044,7 +1065,7 @@
       <c r="Y3"/>
       <c r="Z3" s="2"/>
       <c r="AA3" s="2"/>
-      <c r="AB3" s="9" t="s">
+      <c r="AB3" s="8" t="s">
         <v>41</v>
       </c>
       <c r="AC3" s="1"/>
@@ -1052,38 +1073,38 @@
       <c r="AE3"/>
       <c r="AF3"/>
       <c r="AG3" s="2"/>
-      <c r="AH3" s="8"/>
+      <c r="AH3" s="7"/>
       <c r="AI3"/>
-      <c r="AJ3" s="10"/>
+      <c r="AJ3" s="9"/>
       <c r="AK3" s="2"/>
     </row>
     <row r="4" ht="14.25">
       <c r="A4" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="E4" s="6" t="s">
+      <c r="B4" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="F4" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="H4" s="7" t="s">
+      <c r="F4" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H4" s="6" t="s">
         <v>38</v>
       </c>
       <c r="J4" s="2"/>
-      <c r="K4" s="9" t="s">
+      <c r="K4" s="8" t="s">
         <v>41</v>
       </c>
       <c r="L4" s="2"/>
@@ -1092,7 +1113,7 @@
       <c r="O4" s="1"/>
       <c r="P4"/>
       <c r="Q4"/>
-      <c r="R4" s="8"/>
+      <c r="R4" s="7"/>
       <c r="S4" s="2"/>
       <c r="T4" s="2"/>
       <c r="U4"/>
@@ -1108,7 +1129,7 @@
       <c r="AE4"/>
       <c r="AF4"/>
       <c r="AG4" s="2"/>
-      <c r="AH4" s="9" t="s">
+      <c r="AH4" s="8" t="s">
         <v>41</v>
       </c>
       <c r="AI4"/>
@@ -1119,32 +1140,32 @@
       <c r="A5" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="D5" s="11" t="s">
+      <c r="C5" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="D5" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="E5" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="F5" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="G5" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="H5" s="12" t="s">
+      <c r="E5" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="H5" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="I5" s="13"/>
+      <c r="I5" s="12"/>
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
       <c r="L5" s="3"/>
-      <c r="M5" s="14" t="s">
+      <c r="M5" s="13" t="s">
         <v>41</v>
       </c>
       <c r="N5" s="3"/>
@@ -1152,7 +1173,7 @@
       <c r="P5" s="3"/>
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
-      <c r="S5" s="13"/>
+      <c r="S5" s="12"/>
       <c r="T5" s="3"/>
       <c r="U5" s="3"/>
       <c r="V5" s="4"/>
@@ -1166,7 +1187,7 @@
       <c r="AD5" s="3"/>
       <c r="AE5" s="3"/>
       <c r="AF5" s="3"/>
-      <c r="AG5" s="14" t="s">
+      <c r="AG5" s="13" t="s">
         <v>41</v>
       </c>
       <c r="AH5" s="3"/>
@@ -1186,34 +1207,34 @@
       <c r="A6" t="s">
         <v>45</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E6" s="6" t="s">
+      <c r="B6" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="F6" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="J6" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="K6" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="L6" s="8"/>
+      <c r="F6" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="K6" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="L6" s="7"/>
       <c r="M6" s="2"/>
       <c r="N6"/>
       <c r="O6" s="1"/>
@@ -1232,7 +1253,7 @@
       <c r="AB6"/>
       <c r="AC6" s="1"/>
       <c r="AD6"/>
-      <c r="AE6" s="8"/>
+      <c r="AE6" s="7"/>
       <c r="AF6"/>
       <c r="AG6" s="2"/>
       <c r="AH6" s="2"/>
@@ -1244,25 +1265,25 @@
       <c r="A7" t="s">
         <v>47</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="C7" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="D7" s="6" t="s">
+      <c r="C7" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="E7" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="F7" s="6" t="s">
+      <c r="E7" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G7" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="H7" s="6" t="s">
         <v>39</v>
       </c>
       <c r="J7" s="2"/>
@@ -1284,7 +1305,7 @@
       <c r="Z7" s="2"/>
       <c r="AA7" s="2"/>
       <c r="AB7"/>
-      <c r="AC7" s="15" t="s">
+      <c r="AC7" s="14" t="s">
         <v>41</v>
       </c>
       <c r="AD7"/>
@@ -1293,7 +1314,7 @@
       <c r="AG7" s="2"/>
       <c r="AH7" s="2"/>
       <c r="AI7"/>
-      <c r="AJ7" s="15" t="s">
+      <c r="AJ7" s="14" t="s">
         <v>41</v>
       </c>
       <c r="AK7" s="2"/>
@@ -1302,25 +1323,25 @@
       <c r="A8" t="s">
         <v>48</v>
       </c>
-      <c r="B8" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C8" s="6" t="s">
+      <c r="B8" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="F8" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="H8" s="7" t="s">
+      <c r="F8" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H8" s="6" t="s">
         <v>40</v>
       </c>
       <c r="J8" s="2"/>
@@ -1332,12 +1353,12 @@
       <c r="P8"/>
       <c r="Q8"/>
       <c r="R8"/>
-      <c r="S8" s="8"/>
-      <c r="T8" s="8"/>
+      <c r="S8" s="7"/>
+      <c r="T8" s="7"/>
       <c r="U8"/>
       <c r="V8" s="1"/>
       <c r="W8"/>
-      <c r="X8" s="9" t="s">
+      <c r="X8" s="8" t="s">
         <v>41</v>
       </c>
       <c r="Y8"/>
@@ -1350,7 +1371,7 @@
       <c r="AF8"/>
       <c r="AG8" s="2"/>
       <c r="AH8" s="2"/>
-      <c r="AI8" s="9" t="s">
+      <c r="AI8" s="8" t="s">
         <v>41</v>
       </c>
       <c r="AJ8" s="1"/>
@@ -1360,33 +1381,33 @@
       <c r="A9" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B9" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="F9" s="11" t="s">
+      <c r="B9" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="G9" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="H9" s="12" t="s">
+      <c r="G9" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="H9" s="11" t="s">
         <v>40</v>
       </c>
       <c r="I9" s="3"/>
-      <c r="J9" s="13"/>
-      <c r="K9" s="13"/>
+      <c r="J9" s="12"/>
+      <c r="K9" s="12"/>
       <c r="L9" s="3"/>
       <c r="M9" s="3"/>
-      <c r="N9" s="14" t="s">
+      <c r="N9" s="13" t="s">
         <v>41</v>
       </c>
       <c r="O9" s="4"/>
@@ -1407,7 +1428,7 @@
       <c r="AD9" s="3"/>
       <c r="AE9" s="3"/>
       <c r="AF9" s="3"/>
-      <c r="AG9" s="14" t="s">
+      <c r="AG9" s="13" t="s">
         <v>41</v>
       </c>
       <c r="AH9" s="3"/>
@@ -1428,25 +1449,25 @@
       <c r="A10" t="s">
         <v>50</v>
       </c>
-      <c r="B10" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C10" s="6" t="s">
+      <c r="B10" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D10" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="G10" s="6" t="s">
+      <c r="D10" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="G10" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="H10" s="6" t="s">
         <v>40</v>
       </c>
       <c r="J10" s="2"/>
@@ -1454,62 +1475,109 @@
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
       <c r="N10"/>
-      <c r="O10" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="P10"/>
-      <c r="Q10"/>
-      <c r="R10"/>
-      <c r="S10" s="2"/>
-      <c r="T10" s="2"/>
-      <c r="U10"/>
-      <c r="V10" s="1"/>
-      <c r="W10"/>
-      <c r="X10"/>
-      <c r="Y10"/>
-      <c r="Z10" s="2"/>
-      <c r="AA10" s="2"/>
-      <c r="AB10"/>
-      <c r="AC10" s="1"/>
-      <c r="AD10"/>
-      <c r="AE10"/>
-      <c r="AF10"/>
-      <c r="AG10" s="2"/>
-      <c r="AH10" s="2"/>
-      <c r="AI10"/>
-      <c r="AJ10" s="1"/>
-      <c r="AK10" s="2"/>
+      <c r="O10" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="P10" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q10" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="R10" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="S10" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="T10" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="U10" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="V10" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="W10" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="X10" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="Y10" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="Z10" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="AA10" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB10" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="AC10" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="AD10" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="AE10" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="AF10" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="AG10" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="AH10" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="AI10" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="AJ10" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="AK10" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="AL10" s="15" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="11" ht="14.25">
       <c r="A11" t="s">
         <v>51</v>
       </c>
-      <c r="B11" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="H11" s="7" t="s">
+      <c r="B11" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H11" s="6" t="s">
         <v>46</v>
       </c>
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
       <c r="L11" s="2"/>
-      <c r="M11" s="8"/>
-      <c r="N11" s="9" t="s">
+      <c r="M11" s="7"/>
+      <c r="N11" s="8" t="s">
         <v>41</v>
       </c>
       <c r="O11" s="1"/>
@@ -1518,7 +1586,7 @@
       <c r="R11"/>
       <c r="S11" s="2"/>
       <c r="T11" s="2"/>
-      <c r="U11" s="9" t="s">
+      <c r="U11" s="8" t="s">
         <v>41</v>
       </c>
       <c r="V11" s="1"/>
@@ -1542,29 +1610,29 @@
       <c r="A12" t="s">
         <v>52</v>
       </c>
-      <c r="B12" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" s="6" t="s">
+      <c r="B12" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="E12" s="6" t="s">
+      <c r="D12" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="F12" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G12" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="H12" s="7" t="s">
+      <c r="G12" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="H12" s="6" t="s">
         <v>39</v>
       </c>
       <c r="J12" s="2"/>
-      <c r="K12" s="9" t="s">
+      <c r="K12" s="8" t="s">
         <v>41</v>
       </c>
       <c r="L12" s="2"/>
@@ -1575,18 +1643,18 @@
       <c r="Q12"/>
       <c r="R12"/>
       <c r="S12" s="2"/>
-      <c r="T12" s="8"/>
+      <c r="T12" s="7"/>
       <c r="U12"/>
       <c r="V12" s="1"/>
       <c r="W12"/>
       <c r="X12"/>
       <c r="Y12"/>
-      <c r="Z12" s="9" t="s">
+      <c r="Z12" s="8" t="s">
         <v>41</v>
       </c>
       <c r="AA12" s="2"/>
       <c r="AB12"/>
-      <c r="AC12" s="10"/>
+      <c r="AC12" s="9"/>
       <c r="AD12"/>
       <c r="AE12"/>
       <c r="AF12"/>
@@ -1600,30 +1668,30 @@
       <c r="A13" t="s">
         <v>53</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="C13" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="D13" s="6" t="s">
+      <c r="C13" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="F13" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="G13" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="H13" s="7" t="s">
+      <c r="G13" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H13" s="6" t="s">
         <v>38</v>
       </c>
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
-      <c r="L13" s="9" t="s">
+      <c r="L13" s="8" t="s">
         <v>41</v>
       </c>
       <c r="M13" s="2"/>
@@ -1635,7 +1703,7 @@
       <c r="S13" s="2"/>
       <c r="T13" s="2"/>
       <c r="U13"/>
-      <c r="V13" s="10"/>
+      <c r="V13" s="9"/>
       <c r="W13"/>
       <c r="X13"/>
       <c r="Y13"/>
@@ -1645,7 +1713,7 @@
       <c r="AC13" s="1"/>
       <c r="AD13"/>
       <c r="AE13"/>
-      <c r="AF13" s="9" t="s">
+      <c r="AF13" s="8" t="s">
         <v>41</v>
       </c>
       <c r="AG13" s="2"/>
@@ -1658,27 +1726,55 @@
       <c r="A14" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B14" s="11"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="12"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
-      <c r="M14" s="3"/>
-      <c r="N14" s="3"/>
-      <c r="O14" s="4"/>
+      <c r="B14" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="E14" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="F14" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="G14" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H14" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="I14" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="J14" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="K14" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="L14" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="M14" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="N14" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="O14" s="18" t="s">
+        <v>40</v>
+      </c>
       <c r="P14" s="3"/>
-      <c r="Q14" s="13"/>
+      <c r="Q14" s="12"/>
       <c r="R14" s="3"/>
       <c r="S14" s="3"/>
       <c r="T14" s="3"/>
       <c r="U14" s="3"/>
-      <c r="V14" s="16" t="s">
+      <c r="V14" s="20" t="s">
         <v>41</v>
       </c>
       <c r="W14" s="3"/>
@@ -1687,13 +1783,13 @@
       <c r="Z14" s="3"/>
       <c r="AA14" s="3"/>
       <c r="AB14" s="3"/>
-      <c r="AC14" s="17"/>
+      <c r="AC14" s="21"/>
       <c r="AD14" s="3"/>
       <c r="AE14" s="3"/>
       <c r="AF14" s="3"/>
       <c r="AG14" s="3"/>
       <c r="AH14" s="3"/>
-      <c r="AI14" s="14" t="s">
+      <c r="AI14" s="13" t="s">
         <v>41</v>
       </c>
       <c r="AJ14" s="4"/>
@@ -1711,35 +1807,35 @@
       <c r="A15" t="s">
         <v>55</v>
       </c>
-      <c r="B15" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="G15" s="6" t="s">
+      <c r="B15" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="G15" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="H15" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="I15" s="9" t="s">
+      <c r="H15" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="I15" s="8" t="s">
         <v>41</v>
       </c>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
       <c r="L15" s="2"/>
       <c r="M15" s="2"/>
-      <c r="N15" s="9" t="s">
+      <c r="N15" s="8" t="s">
         <v>41</v>
       </c>
       <c r="O15" s="1"/>
@@ -1770,25 +1866,25 @@
       <c r="A16" t="s">
         <v>56</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D16" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="H16" s="7" t="s">
+      <c r="D16" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="H16" s="6" t="s">
         <v>38</v>
       </c>
       <c r="J16" s="2"/>
@@ -1797,59 +1893,106 @@
       <c r="M16" s="2"/>
       <c r="N16"/>
       <c r="O16" s="1"/>
-      <c r="P16" s="8"/>
-      <c r="Q16"/>
-      <c r="R16"/>
-      <c r="S16" s="2"/>
-      <c r="T16" s="2"/>
-      <c r="U16"/>
-      <c r="V16" s="1"/>
-      <c r="W16"/>
-      <c r="X16"/>
-      <c r="Y16"/>
-      <c r="Z16" s="2"/>
-      <c r="AA16" s="2"/>
-      <c r="AB16"/>
-      <c r="AC16" s="1"/>
-      <c r="AD16"/>
-      <c r="AE16"/>
-      <c r="AF16"/>
-      <c r="AG16" s="2"/>
-      <c r="AH16" s="2"/>
-      <c r="AI16"/>
-      <c r="AJ16" s="1"/>
-      <c r="AK16" s="2"/>
+      <c r="P16" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q16" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="R16" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="S16" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="T16" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="U16" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="V16" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="W16" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="X16" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="Y16" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="Z16" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="AA16" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="AB16" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="AC16" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="AD16" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="AE16" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="AF16" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="AG16" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="AH16" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="AI16" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="AJ16" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="AK16" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="AL16" s="15" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="17" ht="14.25">
       <c r="A17" t="s">
         <v>57</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C17" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="D17" s="6" t="s">
+      <c r="C17" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D17" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="E17" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="F17" s="6" t="s">
+      <c r="E17" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="F17" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="G17" s="6" t="s">
+      <c r="G17" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="H17" s="7" t="s">
+      <c r="H17" s="6" t="s">
         <v>39</v>
       </c>
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
       <c r="L17" s="2"/>
       <c r="M17" s="2"/>
-      <c r="N17" s="9" t="s">
+      <c r="N17" s="8" t="s">
         <v>41</v>
       </c>
       <c r="O17" s="1"/>
@@ -1859,7 +2002,7 @@
       <c r="S17" s="2"/>
       <c r="T17" s="2"/>
       <c r="U17"/>
-      <c r="V17" s="10"/>
+      <c r="V17" s="9"/>
       <c r="W17"/>
       <c r="X17"/>
       <c r="Y17"/>
@@ -1867,7 +2010,7 @@
       <c r="AA17" s="2"/>
       <c r="AB17"/>
       <c r="AC17" s="1"/>
-      <c r="AD17" s="9" t="s">
+      <c r="AD17" s="8" t="s">
         <v>41</v>
       </c>
       <c r="AE17"/>
@@ -1875,32 +2018,32 @@
       <c r="AG17" s="2"/>
       <c r="AH17" s="2"/>
       <c r="AI17"/>
-      <c r="AJ17" s="10"/>
+      <c r="AJ17" s="9"/>
       <c r="AK17" s="2"/>
     </row>
     <row r="18" ht="14.25">
       <c r="A18" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B18" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="E18" s="6" t="s">
+      <c r="B18" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E18" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="F18" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="G18" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="H18" s="7" t="s">
+      <c r="F18" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H18" s="6" t="s">
         <v>40</v>
       </c>
       <c r="I18" s="2"/>
@@ -1908,16 +2051,16 @@
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
       <c r="M18" s="2"/>
-      <c r="N18" s="9"/>
-      <c r="O18" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="P18" s="8"/>
+      <c r="N18" s="8"/>
+      <c r="O18" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="P18" s="7"/>
       <c r="Q18"/>
       <c r="R18"/>
       <c r="S18" s="2"/>
       <c r="T18" s="2"/>
-      <c r="U18" s="9" t="s">
+      <c r="U18" s="8" t="s">
         <v>41</v>
       </c>
       <c r="V18" s="1"/>
@@ -1941,36 +2084,64 @@
       <c r="A19" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B19" s="11"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="12"/>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
-      <c r="K19" s="3"/>
-      <c r="L19" s="3"/>
-      <c r="M19" s="3"/>
-      <c r="N19" s="3"/>
-      <c r="O19" s="4"/>
+      <c r="B19" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="D19" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="E19" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="F19" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="G19" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="H19" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="I19" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="J19" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="K19" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="L19" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="M19" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="N19" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="O19" s="18" t="s">
+        <v>40</v>
+      </c>
       <c r="P19" s="3"/>
       <c r="Q19" s="3"/>
       <c r="R19" s="3"/>
       <c r="S19" s="3"/>
       <c r="T19" s="3"/>
       <c r="U19" s="3"/>
-      <c r="V19" s="17"/>
+      <c r="V19" s="21"/>
       <c r="W19" s="3"/>
       <c r="X19" s="3"/>
       <c r="Y19" s="3"/>
-      <c r="Z19" s="14" t="s">
+      <c r="Z19" s="13" t="s">
         <v>41</v>
       </c>
       <c r="AA19" s="3"/>
       <c r="AB19" s="3"/>
-      <c r="AC19" s="17"/>
+      <c r="AC19" s="21"/>
       <c r="AD19" s="3"/>
       <c r="AE19" s="3"/>
       <c r="AF19" s="3"/>
@@ -1992,31 +2163,31 @@
       <c r="A20" t="s">
         <v>60</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D20" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="F20" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="G20" s="6" t="s">
+      <c r="D20" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G20" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="H20" s="7" t="s">
+      <c r="H20" s="6" t="s">
         <v>46</v>
       </c>
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
       <c r="L20" s="2"/>
-      <c r="M20" s="8"/>
+      <c r="M20" s="7"/>
       <c r="N20"/>
       <c r="O20" s="1"/>
       <c r="P20"/>
@@ -2037,7 +2208,7 @@
       <c r="AE20"/>
       <c r="AF20"/>
       <c r="AG20" s="2"/>
-      <c r="AH20" s="8"/>
+      <c r="AH20" s="7"/>
       <c r="AI20"/>
       <c r="AJ20" s="1"/>
       <c r="AK20" s="2"/>
@@ -2046,25 +2217,25 @@
       <c r="A21" t="s">
         <v>61</v>
       </c>
-      <c r="B21" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="D21" s="6" t="s">
+      <c r="B21" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="E21" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="F21" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G21" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="H21" s="7" t="s">
+      <c r="G21" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="H21" s="6" t="s">
         <v>40</v>
       </c>
       <c r="J21" s="2"/>
@@ -2089,36 +2260,36 @@
       <c r="AC21" s="1"/>
       <c r="AD21"/>
       <c r="AE21"/>
-      <c r="AF21" s="8"/>
+      <c r="AF21" s="7"/>
       <c r="AG21" s="2"/>
       <c r="AH21" s="2"/>
       <c r="AI21"/>
-      <c r="AJ21" s="10"/>
+      <c r="AJ21" s="9"/>
       <c r="AK21" s="2"/>
     </row>
     <row r="22" ht="14.25">
       <c r="A22" t="s">
         <v>62</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D22" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E22" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="F22" s="6" t="s">
+      <c r="D22" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="F22" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G22" s="6" t="s">
+      <c r="G22" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="H22" s="7" t="s">
+      <c r="H22" s="6" t="s">
         <v>46</v>
       </c>
       <c r="J22" s="2"/>
@@ -2131,10 +2302,10 @@
       <c r="Q22"/>
       <c r="R22"/>
       <c r="S22" s="2"/>
-      <c r="T22" s="8"/>
+      <c r="T22" s="7"/>
       <c r="U22"/>
       <c r="V22" s="1"/>
-      <c r="W22" s="8"/>
+      <c r="W22" s="7"/>
       <c r="X22"/>
       <c r="Y22"/>
       <c r="Z22" s="2"/>
@@ -2154,29 +2325,29 @@
       <c r="A23" t="s">
         <v>63</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="D23" s="6" t="s">
+      <c r="B23" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D23" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="E23" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="F23" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="G23" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="H23" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="I23" s="8"/>
-      <c r="J23" s="8"/>
+      <c r="F23" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G23" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="I23" s="7"/>
+      <c r="J23" s="7"/>
       <c r="K23" s="2"/>
       <c r="L23" s="2"/>
       <c r="M23" s="2"/>

</xml_diff>